<commit_message>
Default IFC as of 21-04-2026
</commit_message>
<xml_diff>
--- a/testing_purpose.xlsx
+++ b/testing_purpose.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Divyesh\IFC\AmazonDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C633938-5C11-4694-972D-C2962CCC35DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12270321-E15D-4D9C-98DB-BE5ACFFCA911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="61">
   <si>
     <t>Yes</t>
   </si>
@@ -107,9 +107,6 @@
   </si>
   <si>
     <t>Nature of Control (Preventive or Detective)</t>
-  </si>
-  <si>
-    <t>IPE Reference</t>
   </si>
   <si>
     <t xml:space="preserve">Does the control rely on information produced by the entity?
@@ -258,6 +255,9 @@
   </si>
   <si>
     <t>xyz column</t>
+  </si>
+  <si>
+    <t>abc column</t>
   </si>
 </sst>
 </file>
@@ -562,6 +562,7 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -572,7 +573,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
   <cellStyles count="12">
     <cellStyle name="Comma 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -959,13 +959,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A1" s="46" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
+      <c r="A1" s="47" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
       <c r="D1" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
@@ -995,13 +995,13 @@
       <c r="AD1" s="2"/>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
+      <c r="A2" s="47" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
@@ -1013,7 +1013,7 @@
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
       <c r="N2" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="O2" s="2">
         <v>8</v>
@@ -1035,13 +1035,13 @@
       <c r="AD2" s="2"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A3" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
+      <c r="A3" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
       <c r="D3" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -1053,7 +1053,7 @@
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O3" s="2">
         <v>5</v>
@@ -1107,97 +1107,97 @@
       <c r="AD4" s="2"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A5" s="47" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
+      <c r="A5" s="48" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
       <c r="F5" s="37"/>
-      <c r="G5" s="47" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" s="47"/>
-      <c r="I5" s="47"/>
-      <c r="J5" s="47"/>
-      <c r="K5" s="47"/>
-      <c r="L5" s="45" t="s">
+      <c r="G5" s="48" t="s">
         <v>32</v>
       </c>
-      <c r="M5" s="45"/>
-      <c r="N5" s="45"/>
-      <c r="O5" s="45"/>
-      <c r="P5" s="45"/>
-      <c r="Q5" s="45"/>
-      <c r="R5" s="45"/>
-      <c r="S5" s="45"/>
-      <c r="T5" s="45"/>
-      <c r="U5" s="45"/>
-      <c r="V5" s="45"/>
-      <c r="W5" s="45"/>
-      <c r="X5" s="45"/>
-      <c r="Y5" s="45"/>
-      <c r="Z5" s="45"/>
-      <c r="AA5" s="45"/>
-      <c r="AB5" s="45"/>
-      <c r="AC5" s="45"/>
-      <c r="AD5" s="45"/>
+      <c r="H5" s="48"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="48"/>
+      <c r="K5" s="48"/>
+      <c r="L5" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="M5" s="46"/>
+      <c r="N5" s="46"/>
+      <c r="O5" s="46"/>
+      <c r="P5" s="46"/>
+      <c r="Q5" s="46"/>
+      <c r="R5" s="46"/>
+      <c r="S5" s="46"/>
+      <c r="T5" s="46"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="46"/>
+      <c r="X5" s="46"/>
+      <c r="Y5" s="46"/>
+      <c r="Z5" s="46"/>
+      <c r="AA5" s="46"/>
+      <c r="AB5" s="46"/>
+      <c r="AC5" s="46"/>
+      <c r="AD5" s="46"/>
     </row>
     <row r="6" spans="1:31" s="5" customFormat="1" ht="120.75" x14ac:dyDescent="0.2">
       <c r="A6" s="28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D6" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="28" t="s">
+      <c r="H6" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="28" t="s">
-        <v>55</v>
-      </c>
-      <c r="G6" s="29" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="29" t="s">
-        <v>28</v>
-      </c>
       <c r="I6" s="29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J6" s="29" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K6" s="29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L6" s="28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M6" s="28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="N6" s="28" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O6" s="28" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P6" s="28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="Q6" s="28" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="R6" s="28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="S6" s="28" t="s">
         <v>17</v>
@@ -1215,10 +1215,10 @@
         <v>13</v>
       </c>
       <c r="X6" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y6" s="28" t="s">
         <v>38</v>
-      </c>
-      <c r="Y6" s="28" t="s">
-        <v>39</v>
       </c>
       <c r="Z6" s="41" t="s">
         <v>12</v>
@@ -1236,7 +1236,7 @@
     </row>
     <row r="7" spans="1:31" ht="102" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>5</v>
@@ -1245,16 +1245,16 @@
         <v>4</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E7" s="30" t="s">
         <v>7</v>
       </c>
       <c r="F7" s="30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G7" s="43"/>
-      <c r="H7" s="48" t="s">
+      <c r="H7" s="45" t="s">
         <v>8</v>
       </c>
       <c r="I7" s="43"/>
@@ -1264,22 +1264,22 @@
         <v>6</v>
       </c>
       <c r="M7" s="32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N7" s="32" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="P7" s="16" t="s">
         <v>0</v>
       </c>
       <c r="Q7" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="R7" s="16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="S7" s="17" t="s">
         <v>2</v>
@@ -1291,28 +1291,28 @@
         <v>0</v>
       </c>
       <c r="V7" s="17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="W7" s="17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="X7" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="Y7" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="Z7" s="17" t="s">
         <v>3</v>
       </c>
       <c r="AA7" s="35" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AC7" s="36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AD7" s="42"/>
       <c r="AE7" s="44"/>

</xml_diff>